<commit_message>
commit all updates to all fg and hl tests
</commit_message>
<xml_diff>
--- a/hl_test_results.xlsx
+++ b/hl_test_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -640,6 +640,38 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ICMHULL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2506 23rd St W, Lehigh Acres, FL 33971</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Short-Term Vacant or Unoccupied Dwelling - Basic Form</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>600,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>QB20026611</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>$2,590.25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
committing changes to hl and fg tests
</commit_message>
<xml_diff>
--- a/hl_test_results.xlsx
+++ b/hl_test_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,230 +445,6 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>Premium</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>icmhull</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>15110 Shearcrest Dr, Lithia, FL 33547</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>HO-3</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>800,000</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>QB20026601</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>$3,322.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ICMHULL</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>9607 Bahia Rd, Ocala, FL 34472</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>HO-3 Tenant</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>800,000</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>QB20026602</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>$6,856.40</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ICMHULL</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>7733 Belvoir Dr, Orlando, FL 32835</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>HO Wind Only</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>800,000</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>QB20026603</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>$4,519.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ICMHULL</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1949 Par Dr, Naples, FL 34120</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Short-Term Vacant or Unoccupied Dwelling - Broad Form</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>600,000</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>QB20026605</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>$6,903.65</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ICMHULL</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>3618 Elm St, Ellenton, FL 34222</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Short-Term Vacant or Unoccupied Dwelling - Broad Form</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>600,000</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>QB20026607</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>$3,691.70</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ICMHULL</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>3032 Bridgefield Ct, The Villages, FL 32162</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Short-Term Vacant or Unoccupied Dwelling - Broad Form</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>600,000</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>QB20026610</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>$3,366.20</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ICMHULL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2506 23rd St W, Lehigh Acres, FL 33971</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Short-Term Vacant or Unoccupied Dwelling - Basic Form</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>600,000</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>QB20026611</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>$2,590.25</t>
         </is>
       </c>
     </row>

</xml_diff>